<commit_message>
Update client list (387 contracts) and add 4★/5★ threshold error cards to backtest
Updated client-contracts.xlsx with the April 2026 client list (387 contracts,
up from 257). Added per-threshold error summary cards for the 4-star and 5-star
cut points alongside the existing all-threshold MAE card.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/client-contracts.xlsx
+++ b/data/client-contracts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joshuarenken/Dropbox/Mac/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D345F512-1D9C-5D4A-B840-1EF4EDCD67D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2ADF645C-D975-D845-B06F-1249E7F70A18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1164" uniqueCount="546">
   <si>
     <t>Name</t>
   </si>
@@ -1151,6 +1151,513 @@
   </si>
   <si>
     <t>S5593</t>
+  </si>
+  <si>
+    <t>Blue Cross Blue Shield of Michigan Mutual Ins. Co.</t>
+  </si>
+  <si>
+    <t>Blue Care Network</t>
+  </si>
+  <si>
+    <t>H5883</t>
+  </si>
+  <si>
+    <t>Wellmark Advantage Health Plan</t>
+  </si>
+  <si>
+    <t>H5900</t>
+  </si>
+  <si>
+    <t>NextBlue of North Dakota</t>
+  </si>
+  <si>
+    <t>H6202</t>
+  </si>
+  <si>
+    <t>Vermont Blue Advantage</t>
+  </si>
+  <si>
+    <t>H6898</t>
+  </si>
+  <si>
+    <t>H8095</t>
+  </si>
+  <si>
+    <t>WyoBlue Advantage</t>
+  </si>
+  <si>
+    <t>H9326</t>
+  </si>
+  <si>
+    <t>H9489</t>
+  </si>
+  <si>
+    <t>Blue Cross Blue Shield of Michigan</t>
+  </si>
+  <si>
+    <t>H9572</t>
+  </si>
+  <si>
+    <t>S5584</t>
+  </si>
+  <si>
+    <t>Wellcare</t>
+  </si>
+  <si>
+    <t>H0029</t>
+  </si>
+  <si>
+    <t>Wellcare By Allwell</t>
+  </si>
+  <si>
+    <t>H0062</t>
+  </si>
+  <si>
+    <t>H0074</t>
+  </si>
+  <si>
+    <t>H0111</t>
+  </si>
+  <si>
+    <t>H0174</t>
+  </si>
+  <si>
+    <t>H0270</t>
+  </si>
+  <si>
+    <t>H0351</t>
+  </si>
+  <si>
+    <t>Wellcare By Health Net</t>
+  </si>
+  <si>
+    <t>H0562</t>
+  </si>
+  <si>
+    <t>H0712</t>
+  </si>
+  <si>
+    <t>H0724</t>
+  </si>
+  <si>
+    <t>H0908</t>
+  </si>
+  <si>
+    <t>H0913</t>
+  </si>
+  <si>
+    <t>H1032</t>
+  </si>
+  <si>
+    <t>H1112</t>
+  </si>
+  <si>
+    <t>H1215</t>
+  </si>
+  <si>
+    <t>H1395</t>
+  </si>
+  <si>
+    <t>H1416</t>
+  </si>
+  <si>
+    <t>H1664</t>
+  </si>
+  <si>
+    <t>H1862</t>
+  </si>
+  <si>
+    <t>H1914</t>
+  </si>
+  <si>
+    <t>H2117</t>
+  </si>
+  <si>
+    <t>H2162</t>
+  </si>
+  <si>
+    <t>Wellcare By Trillium</t>
+  </si>
+  <si>
+    <t>H2174</t>
+  </si>
+  <si>
+    <t>H2491</t>
+  </si>
+  <si>
+    <t>H2775</t>
+  </si>
+  <si>
+    <t>H2816</t>
+  </si>
+  <si>
+    <t>Ascension Complete</t>
+  </si>
+  <si>
+    <t>H2853</t>
+  </si>
+  <si>
+    <t>H3499</t>
+  </si>
+  <si>
+    <t>H3561</t>
+  </si>
+  <si>
+    <t>H3975</t>
+  </si>
+  <si>
+    <t>H4073</t>
+  </si>
+  <si>
+    <t>H4158</t>
+  </si>
+  <si>
+    <t>H4506</t>
+  </si>
+  <si>
+    <t>H4537</t>
+  </si>
+  <si>
+    <t>H4661</t>
+  </si>
+  <si>
+    <t>H4847</t>
+  </si>
+  <si>
+    <t>H4868</t>
+  </si>
+  <si>
+    <t>H5087</t>
+  </si>
+  <si>
+    <t>H5117</t>
+  </si>
+  <si>
+    <t>H5190</t>
+  </si>
+  <si>
+    <t>Wellcare By Absolute Total Care</t>
+  </si>
+  <si>
+    <t>H5272</t>
+  </si>
+  <si>
+    <t>H5294</t>
+  </si>
+  <si>
+    <t>H5439</t>
+  </si>
+  <si>
+    <t>H5475</t>
+  </si>
+  <si>
+    <t>H5590</t>
+  </si>
+  <si>
+    <t>Wellcare By Fidelis Care</t>
+  </si>
+  <si>
+    <t>H5599</t>
+  </si>
+  <si>
+    <t>H5779</t>
+  </si>
+  <si>
+    <t>H5965</t>
+  </si>
+  <si>
+    <t>H6348</t>
+  </si>
+  <si>
+    <t>H6550</t>
+  </si>
+  <si>
+    <t>H6815</t>
+  </si>
+  <si>
+    <t>Wellcare By Meridian</t>
+  </si>
+  <si>
+    <t>H6971</t>
+  </si>
+  <si>
+    <t>H7323</t>
+  </si>
+  <si>
+    <t>H7326</t>
+  </si>
+  <si>
+    <t>H7435</t>
+  </si>
+  <si>
+    <t>H7512</t>
+  </si>
+  <si>
+    <t>H7518</t>
+  </si>
+  <si>
+    <t>H8121</t>
+  </si>
+  <si>
+    <t>Wellcare by Allwell</t>
+  </si>
+  <si>
+    <t>H8189</t>
+  </si>
+  <si>
+    <t>H8711</t>
+  </si>
+  <si>
+    <t>H9364</t>
+  </si>
+  <si>
+    <t>H9387</t>
+  </si>
+  <si>
+    <t>H9630</t>
+  </si>
+  <si>
+    <t>H9730</t>
+  </si>
+  <si>
+    <t>H9811</t>
+  </si>
+  <si>
+    <t>H9916</t>
+  </si>
+  <si>
+    <t>S4802</t>
+  </si>
+  <si>
+    <t>Elevance Health, Inc.</t>
+  </si>
+  <si>
+    <t>Anthem Blue Cross</t>
+  </si>
+  <si>
+    <t>H0544</t>
+  </si>
+  <si>
+    <t>Anthem Blue Cross and Blue Shield</t>
+  </si>
+  <si>
+    <t>H0629</t>
+  </si>
+  <si>
+    <t>Wellpoint</t>
+  </si>
+  <si>
+    <t>H0907</t>
+  </si>
+  <si>
+    <t>H1212</t>
+  </si>
+  <si>
+    <t>H1423</t>
+  </si>
+  <si>
+    <t>H1607</t>
+  </si>
+  <si>
+    <t>H1894</t>
+  </si>
+  <si>
+    <t>Healthy Blue</t>
+  </si>
+  <si>
+    <t>H1947</t>
+  </si>
+  <si>
+    <t>H2441</t>
+  </si>
+  <si>
+    <t>H2593</t>
+  </si>
+  <si>
+    <t>H2628</t>
+  </si>
+  <si>
+    <t>H2687</t>
+  </si>
+  <si>
+    <t>H2836</t>
+  </si>
+  <si>
+    <t>H3240</t>
+  </si>
+  <si>
+    <t>Anthem HealthKeepers</t>
+  </si>
+  <si>
+    <t>H3447</t>
+  </si>
+  <si>
+    <t>H3536</t>
+  </si>
+  <si>
+    <t>H3655</t>
+  </si>
+  <si>
+    <t>Medicare y Mucho Mas (MMM)</t>
+  </si>
+  <si>
+    <t>H4003</t>
+  </si>
+  <si>
+    <t>H4004</t>
+  </si>
+  <si>
+    <t>H4036</t>
+  </si>
+  <si>
+    <t>Anthem Blue Cross Partnership Plan</t>
+  </si>
+  <si>
+    <t>H4161</t>
+  </si>
+  <si>
+    <t>H4346</t>
+  </si>
+  <si>
+    <t>H4471</t>
+  </si>
+  <si>
+    <t>H4694</t>
+  </si>
+  <si>
+    <t>Anthem Blue Cross Life and Health Insurance Compan</t>
+  </si>
+  <si>
+    <t>H4704</t>
+  </si>
+  <si>
+    <t>H4909</t>
+  </si>
+  <si>
+    <t>H5422</t>
+  </si>
+  <si>
+    <t>Freedom Health, Inc.</t>
+  </si>
+  <si>
+    <t>H5427</t>
+  </si>
+  <si>
+    <t>HealthSun Health Plans, Inc.</t>
+  </si>
+  <si>
+    <t>H5431</t>
+  </si>
+  <si>
+    <t>Simply Healthcare Plans, Inc.</t>
+  </si>
+  <si>
+    <t>H5471</t>
+  </si>
+  <si>
+    <t>Optimum HealthCare, Inc.</t>
+  </si>
+  <si>
+    <t>H5594</t>
+  </si>
+  <si>
+    <t>H5828</t>
+  </si>
+  <si>
+    <t>H5854</t>
+  </si>
+  <si>
+    <t>Blue Medicare Advantage</t>
+  </si>
+  <si>
+    <t>H6078</t>
+  </si>
+  <si>
+    <t>H6316</t>
+  </si>
+  <si>
+    <t>Anthem Blue Cross and Blue Shield HP</t>
+  </si>
+  <si>
+    <t>H6988</t>
+  </si>
+  <si>
+    <t>H7093</t>
+  </si>
+  <si>
+    <t>H7220</t>
+  </si>
+  <si>
+    <t>H7522</t>
+  </si>
+  <si>
+    <t>H8432</t>
+  </si>
+  <si>
+    <t>H8552</t>
+  </si>
+  <si>
+    <t>H8849</t>
+  </si>
+  <si>
+    <t>AMH Health</t>
+  </si>
+  <si>
+    <t>H9065</t>
+  </si>
+  <si>
+    <t>H9219</t>
+  </si>
+  <si>
+    <t>H9525</t>
+  </si>
+  <si>
+    <t>R5941</t>
+  </si>
+  <si>
+    <t>Elevance Health, Inc. &amp; BCBSMA &amp; BCBSRI &amp; BCBSVT</t>
+  </si>
+  <si>
+    <t>Blue MedicareRx</t>
+  </si>
+  <si>
+    <t>S2893</t>
+  </si>
+  <si>
+    <t>Anthem Insurance Companies, Inc.</t>
+  </si>
+  <si>
+    <t>S5596</t>
+  </si>
+  <si>
+    <t>S5960</t>
+  </si>
+  <si>
+    <t>UPMC Health System</t>
+  </si>
+  <si>
+    <t>UPMC for Life</t>
+  </si>
+  <si>
+    <t>H3907</t>
+  </si>
+  <si>
+    <t>UPMC for Life Complete Care</t>
+  </si>
+  <si>
+    <t>H4279</t>
+  </si>
+  <si>
+    <t>H5533</t>
+  </si>
+  <si>
+    <t>H7123</t>
+  </si>
+  <si>
+    <t>UPMC Health Plan</t>
+  </si>
+  <si>
+    <t>S3389</t>
   </si>
 </sst>
 </file>
@@ -1544,7 +2051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C259"/>
+  <dimension ref="A1:C389"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -2610,7 +3117,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>191</v>
       </c>
@@ -2621,7 +3128,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
         <v>195</v>
       </c>
@@ -4390,6 +4897,1436 @@
       </c>
       <c r="C259" s="1" t="s">
         <v>376</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A260" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B260" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C260" s="1" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="261" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A261" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B261" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="C261" s="1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A262" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B262" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="C262" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A263" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B263" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="C263" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="264" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A264" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B264" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="C264" s="1" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A265" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B265" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="C265" s="1" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A266" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B266" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="C266" s="1" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A267" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B267" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C267" s="1" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="268" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A268" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B268" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C268" s="1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A269" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B269" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C269" s="1" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="270" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A270" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B270" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C270" s="1" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A271" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B271" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C271" s="1" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="272" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A272" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B272" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C272" s="1" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A273" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B273" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C273" s="1" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="274" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A274" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B274" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C274" s="1" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="275" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A275" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B275" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C275" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A276" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B276" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="C276" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="277" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A277" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B277" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C277" s="1" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A278" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B278" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C278" s="1" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="279" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A279" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B279" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C279" s="1" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="280" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A280" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B280" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C280" s="1" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A281" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B281" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C281" s="1" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A282" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B282" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C282" s="1" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="283" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A283" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B283" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C283" s="1" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="284" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A284" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B284" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C284" s="1" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="285" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A285" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B285" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C285" s="1" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A286" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C286" s="1" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A287" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B287" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C287" s="1" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A288" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B288" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C288" s="1" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="289" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A289" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B289" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C289" s="1" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="290" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A290" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C290" s="1" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="291" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A291" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="C291" s="1" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="292" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A292" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C292" s="1" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="293" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A293" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B293" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C293" s="1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="294" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A294" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C294" s="1" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="295" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A295" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="C295" s="1" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="296" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A296" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C296" s="1" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A297" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B297" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="C297" s="1" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A298" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B298" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C298" s="1" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A299" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B299" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C299" s="1" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A300" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B300" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C300" s="1" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A301" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B301" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C301" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A302" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B302" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C302" s="1" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A303" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B303" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C303" s="1" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A304" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B304" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C304" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A305" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B305" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C305" s="1" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A306" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B306" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C306" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A307" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B307" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C307" s="1" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A308" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B308" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C308" s="1" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A309" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B309" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="C309" s="1" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A310" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B310" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C310" s="1" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A311" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B311" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="C311" s="1" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A312" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B312" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C312" s="1" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A313" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B313" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C313" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A314" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B314" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="C314" s="1" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A315" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B315" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C315" s="1" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A316" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B316" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C316" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A317" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B317" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C317" s="1" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A318" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B318" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C318" s="1" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A319" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B319" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="C319" s="1" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A320" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B320" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C320" s="1" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="321" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A321" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B321" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C321" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A322" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B322" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C322" s="1" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="323" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A323" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B323" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C323" s="1" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="324" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A324" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B324" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="C324" s="1" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="325" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A325" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B325" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C325" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="326" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A326" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B326" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="C326" s="1" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="327" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A327" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B327" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="C327" s="1" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A328" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B328" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C328" s="1" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="329" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A329" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B329" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C329" s="1" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="330" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A330" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B330" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C330" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="331" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A331" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B331" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C331" s="1" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="332" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A332" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B332" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C332" s="1" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="333" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A333" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B333" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C333" s="1" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="334" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A334" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B334" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C334" s="1" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="335" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A335" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B335" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C335" s="1" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="336" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A336" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B336" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="C336" s="1" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="337" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A337" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B337" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C337" s="1" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="338" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A338" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B338" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C338" s="1" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="339" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A339" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B339" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C339" s="1" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="340" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A340" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B340" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C340" s="1" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="341" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A341" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B341" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C341" s="1" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="342" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A342" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B342" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C342" s="1" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="343" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A343" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B343" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="C343" s="1" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="344" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A344" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B344" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C344" s="1" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="345" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A345" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B345" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C345" s="1" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="346" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A346" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B346" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C346" s="1" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A347" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B347" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C347" s="1" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="348" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A348" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B348" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C348" s="1" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="349" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A349" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B349" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C349" s="1" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A350" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B350" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="C350" s="1" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="351" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A351" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B351" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C351" s="1" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="352" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A352" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B352" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C352" s="1" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="353" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A353" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B353" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="C353" s="1" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="354" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A354" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B354" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="C354" s="1" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="355" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A355" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B355" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C355" s="1" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="356" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A356" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B356" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="C356" s="1" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="357" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A357" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B357" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C357" s="1" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="358" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A358" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B358" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="C358" s="1" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="359" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A359" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B359" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="C359" s="1" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="360" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A360" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B360" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="C360" s="1" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="361" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A361" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B361" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C361" s="1" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="362" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A362" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B362" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C362" s="1" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="363" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A363" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B363" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="C363" s="1" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="364" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A364" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B364" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="C364" s="1" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="365" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A365" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B365" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="C365" s="1" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="366" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A366" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B366" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="C366" s="1" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="367" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A367" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B367" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C367" s="1" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="368" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A368" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B368" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C368" s="1" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="369" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A369" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B369" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="C369" s="1" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="370" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A370" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B370" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="C370" s="1" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="371" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A371" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B371" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="C371" s="1" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="372" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A372" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B372" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C372" s="1" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="373" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A373" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B373" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="C373" s="1" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="374" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A374" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B374" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="C374" s="1" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="375" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A375" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B375" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="C375" s="1" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="376" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A376" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B376" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="C376" s="1" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="377" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A377" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B377" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C377" s="1" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="378" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A378" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B378" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="C378" s="1" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="379" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A379" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B379" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="C379" s="1" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="380" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A380" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B380" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C380" s="1" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="381" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A381" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B381" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C381" s="1" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="382" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A382" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="B382" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="C382" s="1" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="383" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A383" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B383" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="C383" s="1" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="384" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A384" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B384" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C384" s="1" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="385" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A385" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="B385" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="C385" s="1" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="386" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A386" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="B386" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="C386" s="1" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="387" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A387" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="B387" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="C387" s="1" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="388" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A388" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="B388" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="C388" s="1" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="389" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A389" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="B389" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="C389" s="1" t="s">
+        <v>545</v>
       </c>
     </row>
   </sheetData>

</xml_diff>